<commit_message>
add exams and tests
</commit_message>
<xml_diff>
--- a/05_exams/0_fastapi/questions_en.xlsx
+++ b/05_exams/0_fastapi/questions_en.xlsx
@@ -1,19 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="questions" sheetId="1" r:id="rId4"/>
+    <sheet r:id="rId1" sheetId="1" name="questions"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">questions!$A$1:$Z$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">questions!$A$1:$Z$77</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="310">
   <si>
     <t>question</t>
   </si>
@@ -208,6 +212,12 @@
   </si>
   <si>
     <t>Data Streaming</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
   <si>
     <t>Kafka is messaging system</t>
@@ -943,23 +953,21 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -967,52 +975,88 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFffffff"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="3">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFc6c6c6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFc6c6c6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFc6c6c6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="6">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -1039,22 +1083,82 @@
         <a:srgbClr val="46BDC6"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1066,156 +1170,187 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:tint val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="9500"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot rev="0" lon="0" lat="0"/>
+            </a:camera>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:tint val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF1E824C"/>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I77"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="107.75"/>
-    <col customWidth="1" min="2" max="2" width="17.75"/>
-    <col customWidth="1" min="3" max="3" width="18.13"/>
-    <col customWidth="1" min="5" max="5" width="82.0"/>
-    <col customWidth="1" min="6" max="6" width="118.0"/>
-    <col customWidth="1" min="7" max="8" width="78.38"/>
-    <col customWidth="1" min="9" max="9" width="10.38"/>
+    <col min="1" max="1" style="5" width="107.7192857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="17.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="82.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="118.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="78.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="78.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="10.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1244,7 +1379,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -1266,8 +1401,10 @@
       <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -1292,8 +1429,9 @@
       <c r="H3" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="I3" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1318,8 +1456,9 @@
       <c r="H4" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="I4" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -1344,8 +1483,9 @@
       <c r="H5" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="I5" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1367,8 +1507,10 @@
       <c r="G6" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
@@ -1393,8 +1535,9 @@
       <c r="H7" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="I7" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -1416,8 +1559,10 @@
       <c r="G8" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="9">
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
         <v>40</v>
       </c>
@@ -1439,8 +1584,10 @@
       <c r="G9" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10">
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
@@ -1462,8 +1609,10 @@
       <c r="G10" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
         <v>48</v>
       </c>
@@ -1485,8 +1634,10 @@
       <c r="G11" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="12">
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
         <v>50</v>
       </c>
@@ -1508,8 +1659,10 @@
       <c r="G12" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="13">
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
         <v>54</v>
       </c>
@@ -1531,8 +1684,10 @@
       <c r="G13" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="14">
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
         <v>58</v>
       </c>
@@ -1557,8 +1712,9 @@
       <c r="H14" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="15">
+      <c r="I14" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
         <v>63</v>
       </c>
@@ -1571,16 +1727,19 @@
       <c r="D15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
+      <c r="E15" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>64</v>
@@ -1592,21 +1751,22 @@
         <v>25</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="17">
+      <c r="I16" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>64</v>
@@ -1618,24 +1778,25 @@
         <v>25</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="18">
+      <c r="I17" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>11</v>
@@ -1644,21 +1805,23 @@
         <v>12</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F18" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>11</v>
@@ -1667,21 +1830,23 @@
         <v>17</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>83</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>11</v>
@@ -1690,21 +1855,23 @@
         <v>23</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>87</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>11</v>
@@ -1713,21 +1880,23 @@
         <v>17</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>91</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>11</v>
@@ -1736,1321 +1905,1419 @@
         <v>12</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>91</v>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="C24" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F24" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="B25" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>106</v>
+      </c>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>109</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>113</v>
+      </c>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>117</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>120</v>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>123</v>
+      </c>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>127</v>
+      </c>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>127</v>
+      </c>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H33" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="34">
+      <c r="I33" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="35">
+      <c r="I34" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="36">
+      <c r="I35" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="37">
+      <c r="I36" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="I37" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+      <c r="A38" s="4" t="s">
+        <v>147</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>150</v>
+      </c>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>154</v>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>158</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="42">
+      <c r="I41" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="43">
+      <c r="I42" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+      <c r="A44" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>175</v>
+      </c>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>181</v>
+      </c>
+      <c r="I45" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>185</v>
+      </c>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>190</v>
+      </c>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>197</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>200</v>
+      </c>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>203</v>
+      </c>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F51" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="I51" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+      <c r="A52" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="G51" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="H51" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>203</v>
-      </c>
       <c r="C52" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>214</v>
+      </c>
+      <c r="I52" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
       <c r="A53" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B53" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="F53" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="54">
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
       <c r="A54" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>219</v>
+      </c>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
       <c r="A55" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>222</v>
+      </c>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
       <c r="A56" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>226</v>
+      </c>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
       <c r="A57" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>230</v>
+      </c>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
       <c r="A58" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="59">
+      <c r="I58" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
       <c r="A59" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>240</v>
+      </c>
+      <c r="I59" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
       <c r="A60" s="1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H60" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="61">
+      <c r="I60" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="62">
+        <v>249</v>
+      </c>
+      <c r="I61" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
       <c r="A62" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="63">
+        <v>253</v>
+      </c>
+      <c r="I62" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
       <c r="A63" s="1" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>253</v>
+      </c>
+      <c r="I63" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
       <c r="A64" s="1" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>259</v>
+      </c>
+      <c r="I64" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
       <c r="A65" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H65" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="66">
+      <c r="I65" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
       <c r="A66" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H66" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="67">
+      <c r="I66" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
       <c r="A67" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H67" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="68">
+      <c r="I67" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
       <c r="A68" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>271</v>
+      </c>
+      <c r="H68" s="2"/>
+      <c r="I68" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
       <c r="A69" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="70">
+        <v>276</v>
+      </c>
+      <c r="I69" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
       <c r="A70" s="1" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D70" s="2"/>
       <c r="E70" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="71">
+        <v>281</v>
+      </c>
+      <c r="I70" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
       <c r="A71" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D71" s="2"/>
       <c r="E71" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="72">
+        <v>285</v>
+      </c>
+      <c r="H71" s="2"/>
+      <c r="I71" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
       <c r="A72" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D72" s="2"/>
       <c r="E72" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H72" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="73">
+      <c r="I72" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
       <c r="A73" s="1" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D73" s="2"/>
       <c r="E73" s="1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="74">
+        <v>294</v>
+      </c>
+      <c r="I73" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
       <c r="A74" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D74" s="2"/>
       <c r="E74" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>298</v>
+      </c>
+      <c r="H74" s="2"/>
+      <c r="I74" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
       <c r="A75" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D75" s="2"/>
       <c r="E75" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="76">
+        <v>301</v>
+      </c>
+      <c r="G75" s="2"/>
+      <c r="H75" s="2"/>
+      <c r="I75" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
       <c r="A76" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D76" s="2"/>
       <c r="E76" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H76" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="77">
+      <c r="I76" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
       <c r="A77" s="1" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="D77" s="2"/>
       <c r="E77" s="1" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>307</v>
-      </c>
+        <v>309</v>
+      </c>
+      <c r="H77" s="2"/>
+      <c r="I77" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$Z$77"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>